<commit_message>
Auto backup 2026-06-30 11:05:01
</commit_message>
<xml_diff>
--- a/SwissTechMohsin/Listing All Details/02-06-2026/Camera Final.xlsx
+++ b/SwissTechMohsin/Listing All Details/02-06-2026/Camera Final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0dd4d47be472dfe3/Desktop/Listing All Details/02-06-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Listing All Details\02-06-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="640" documentId="8_{06451FDD-92AB-4F11-ADC0-5DCA2BA468F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5578E2A4-D3A5-4BB2-90D5-4836BC2D6530}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{71EB1AA8-6482-4BA1-AE11-C94B0398C988}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{71EB1AA8-6482-4BA1-AE11-C94B0398C988}"/>
   </bookViews>
   <sheets>
     <sheet name="Camera" sheetId="1" r:id="rId1"/>
@@ -770,10 +770,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>